<commit_message>
Fetching solely block in naver
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zasq1\python\fetch\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A235387-F886-4396-A9AF-C06C8200FBCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6D41C04-1849-4F53-9DEC-0DCC10FFD02B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{5131C180-DAEC-4611-8C10-8AAAE970FE8B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="128">
   <si>
     <t>아기이나는시기</t>
   </si>
@@ -45,24 +45,6 @@
   </si>
   <si>
     <t>당체크</t>
-  </si>
-  <si>
-    <t>https://in.naver.com/stevenlove/contents/internal/903509442260352?areacode=itb_bas%2Af_challenge&amp;query=%EC%95%84%EA%B8%B0%EC%9D%B4%EB%82%98%EB%8A%94%EC%8B%9C%EA%B8%B0</t>
-  </si>
-  <si>
-    <t>아기이나는시기 이나는순서</t>
-  </si>
-  <si>
-    <t>https://in.naver.com/eunchoda/contents/internal/903851176578464?areacode=itb_bas%2Af_challenge&amp;query=%EB%B9%88%ED%98%88%EC%97%90%EC%A2%8B%EC%9D%80%EC%9D%8C%EC%8B%9D</t>
-  </si>
-  <si>
-    <t>빈혈에좋은음식 원인 증상! 영양밸런스 이것?</t>
-  </si>
-  <si>
-    <t>https://in.naver.com/binaida/contents/internal/895345180228704?areacode=ink*a&amp;query=%ED%98%88%EB%8B%B9%EC%A1%B0%EC%A0%88</t>
-  </si>
-  <si>
-    <t>혈당조절 당체크 적신호라면? 관리 시작할 때!</t>
   </si>
   <si>
     <t>keyword</t>
@@ -72,16 +54,373 @@
     <t>아기성장발달</t>
   </si>
   <si>
-    <t>https://in.naver.com/allcllrp/contents/internal/897498796699040?areacode=itb_bas%2Af_challenge&amp;query=%EC%95%84%EA%B8%B0%EC%84%B1%EC%9E%A5%EB%B0%9C%EB%8B%AC</t>
-  </si>
-  <si>
-    <t>아기성장발달 아기배밀이시기와 아기기는시기</t>
-  </si>
-  <si>
     <t>target_url</t>
   </si>
   <si>
     <t>target_title</t>
+  </si>
+  <si>
+    <t>당뇨정상수치 전조증상 초기증상</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/binaida/contents/internal/896756059905280?areacode=itb_bas%2Af_challenge&amp;query=%EC%B2%A0%EA%B2%B0%ED%95%8D%EC%84%B1%EB%B9%88%ED%98%88</t>
+  </si>
+  <si>
+    <t>철결핍성빈혈 기립성 '자가진단' 및 대응방법!</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/fff1503/contents/internal/902401441615488?areacode=ink*a&amp;query=%EC%97%BC%EC%A6%9D%EC%A3%BC%EC%82%AC</t>
+  </si>
+  <si>
+    <t>염증주사 염증약 먹고도 재발? 반드시 신경 쓸 것은</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/fff1503/contents/internal/896759474687296?areacode=ink*a&amp;query=%EC%B2%A0%EB%B6%84%EC%A0%9C%EB%B3%B5%EC%9A%A9%EB%B2%95</t>
+  </si>
+  <si>
+    <t>철분제복용법 철분부족 대처법</t>
+  </si>
+  <si>
+    <t>혈압낮추는법</t>
+  </si>
+  <si>
+    <t>갱년기영양제</t>
+  </si>
+  <si>
+    <t>여성갱년기증상</t>
+  </si>
+  <si>
+    <t>흑염소진액효능</t>
+  </si>
+  <si>
+    <t>흑염소즙효능</t>
+  </si>
+  <si>
+    <t>염소즙효능</t>
+  </si>
+  <si>
+    <t>아기기는시기</t>
+  </si>
+  <si>
+    <t>배밀이시기</t>
+  </si>
+  <si>
+    <t>아기배밀이시기</t>
+  </si>
+  <si>
+    <t>아기이나는순서</t>
+  </si>
+  <si>
+    <t>당뇨정상수치</t>
+  </si>
+  <si>
+    <t>혈당관리</t>
+  </si>
+  <si>
+    <t>고혈압증상</t>
+  </si>
+  <si>
+    <t>빈혈증상</t>
+  </si>
+  <si>
+    <t>빈혈원인</t>
+  </si>
+  <si>
+    <t>유아영양제</t>
+  </si>
+  <si>
+    <t>유아비타민</t>
+  </si>
+  <si>
+    <t>유아오메가3</t>
+  </si>
+  <si>
+    <t>울금효능</t>
+  </si>
+  <si>
+    <t>울금강황</t>
+  </si>
+  <si>
+    <t>몸속염증제거</t>
+  </si>
+  <si>
+    <t>만성염증증상</t>
+  </si>
+  <si>
+    <t>만성편도염</t>
+  </si>
+  <si>
+    <t>혈당조절</t>
+  </si>
+  <si>
+    <t>철결핍성빈혈</t>
+  </si>
+  <si>
+    <t>기립성빈혈</t>
+  </si>
+  <si>
+    <t>빈혈자가진단</t>
+  </si>
+  <si>
+    <t>혈당낮추는법</t>
+  </si>
+  <si>
+    <t>혈당영양제</t>
+  </si>
+  <si>
+    <t>남자갱년기증상</t>
+  </si>
+  <si>
+    <t>남성갱년기영양제</t>
+  </si>
+  <si>
+    <t>남성갱년기증상</t>
+  </si>
+  <si>
+    <t>테스토스테론</t>
+  </si>
+  <si>
+    <t>남성호르몬</t>
+  </si>
+  <si>
+    <t>무릎통증</t>
+  </si>
+  <si>
+    <t>무릎염증</t>
+  </si>
+  <si>
+    <t>무릎소리</t>
+  </si>
+  <si>
+    <t>커큐민효능</t>
+  </si>
+  <si>
+    <t>강황의효능</t>
+  </si>
+  <si>
+    <t>스트레스성위염</t>
+  </si>
+  <si>
+    <t>염증주사</t>
+  </si>
+  <si>
+    <t>염증약</t>
+  </si>
+  <si>
+    <t>항산화영양제</t>
+  </si>
+  <si>
+    <t>항산화식품</t>
+  </si>
+  <si>
+    <t>철분제복용법</t>
+  </si>
+  <si>
+    <t>철분부족</t>
+  </si>
+  <si>
+    <t>어지러움증상</t>
+  </si>
+  <si>
+    <t>어지러움약</t>
+  </si>
+  <si>
+    <t>골다공증에좋은음식</t>
+  </si>
+  <si>
+    <t>골감소증</t>
+  </si>
+  <si>
+    <t>에스트로겐영양제</t>
+  </si>
+  <si>
+    <t>폐경증상</t>
+  </si>
+  <si>
+    <t>간기능개선제</t>
+  </si>
+  <si>
+    <t>간기능저하</t>
+  </si>
+  <si>
+    <t>간보호제</t>
+  </si>
+  <si>
+    <t>간영양제</t>
+  </si>
+  <si>
+    <t>밀크씨슬효능</t>
+  </si>
+  <si>
+    <t>간건강</t>
+  </si>
+  <si>
+    <t>간영양제추천</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/binaida/contents/internal/906716805184896?areacode=itb_bas%2Af_challenge&amp;query=%ED%85%8C%EC%8A%A4%ED%86%A0%EC%8A%A4%ED%85%8C%EB%A1%A0</t>
+  </si>
+  <si>
+    <t>테스토스테론 남성호르몬 떨어질 때 관리 방법 요령!</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/livinghealth365/contents/internal/906710345321792?areacode=ink*a&amp;query=%EB%AC%B4%EB%A6%8E%ED%86%B5%EC%A6%9D</t>
+  </si>
+  <si>
+    <t>무릎통증 염증 소리 원인 이유 증상 관리 대처법!</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/livinghealth365/contents/internal/906700290489344?areacode=itb_bas%2Af_challenge&amp;query=%EA%B0%84%EC%98%81%EC%96%91%EC%A0%9C</t>
+  </si>
+  <si>
+    <t>간영양제 추천 밀크씨슬효능 간건강 충분할까?</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/fff1503/contents/internal/906868509736160?areacode=ink*a&amp;query=%EC%8A%A4%ED%8A%B8%EB%A0%88%EC%8A%A4%EC%84%B1%EC%9C%84%EC%97%BC</t>
+  </si>
+  <si>
+    <t>스트레스성위염 신경성위염 증상 반복 원인, 위복합 관리법</t>
+  </si>
+  <si>
+    <t>신경성위염</t>
+  </si>
+  <si>
+    <t>염증수치</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/allcllrp/contents/internal/906881920998720?areacode=itb_bas%2Af_challenge&amp;query=%EA%B0%B1%EB%85%84%EA%B8%B0%EC%98%81%EC%96%91%EC%A0%9C</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/livinghealth365/contents/internal/907066478153376?areacode=ink*a&amp;query=%EB%82%A8%EC%9E%90%EA%B0%B1%EB%85%84%EA%B8%B0%EC%A6%9D%EC%83%81</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/fff1503/contents/internal/907366863011136?areacode=ink*a&amp;query=%EC%96%B4%EC%A7%80%EB%9F%AC%EC%9B%80%EC%A6%9D%EC%83%81</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/sjsjno2/contents/internal/907255760313984?areacode=ink*a&amp;query=%EC%97%90%EC%8A%A4%ED%8A%B8%EB%A1%9C%EA%B2%90%EC%98%81%EC%96%91%EC%A0%9C</t>
+  </si>
+  <si>
+    <t>여성 여자갱년기증상 갱년기영양제!</t>
+  </si>
+  <si>
+    <t>남자갱년기증상 남성 관리하는 갱년기영양제 가이드</t>
+  </si>
+  <si>
+    <t>어지러움증상 반복되는 원인, 어지러움약 선택 전 확인할 점</t>
+  </si>
+  <si>
+    <t>에스트로겐영양제 핵심 기준 폐경증상 관리를 위한 선택</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/binaida/contents/internal/907404973374656?areacode=itb_bas%2Af_challenge&amp;query=%EC%9A%B8%EA%B8%88%ED%9A%A8%EB%8A%A5</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/allcllrp/contents/internal/907605980671296?areacode=ink*a&amp;query=%EB%8B%B9%EB%87%A8%EC%A0%95%EC%83%81%EC%88%98%EC%B9%98</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/binaida/contents/internal/908337175575520?areacode=ink*a&amp;query=%ED%98%88%EB%8B%B9%EC%A1%B0%EC%A0%88</t>
+  </si>
+  <si>
+    <t>혈당조절 실패 이유, 당체크 전 반드시 체크할 사항!</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/stevenlove/contents/internal/907064474160416?areacode=ink*a&amp;query=%EC%95%84%EA%B8%B0%EC%9D%B4%EB%82%98%EB%8A%94%EC%8B%9C%EA%B8%B0</t>
+  </si>
+  <si>
+    <t>아기이나는시기와 아기기는시기 정리!!</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/daily_sossin/contents/internal/909002450460352?areacode=itb_bas%2Af_challenge&amp;query=%EC%BB%A4%ED%81%90%EB%AF%BC%ED%9A%A8%EB%8A%A5</t>
+  </si>
+  <si>
+    <t>커큐민효능 강황의효능 과학적 근거 및 활용법</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/fff1503/contents/internal/909137944145248?areacode=itb_bas%2Af_challenge&amp;query=%ED%95%AD%EC%82%B0%ED%99%94%EC%98%81%EC%96%91%EC%A0%9C</t>
+  </si>
+  <si>
+    <t>항산화영양제 항산화식품 흡수율까지 고려한 항산화 관리법</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/sjsjno2/contents/internal/909022990200000?areacode=itb_bas%2Af_challenge&amp;query=%EA%B3%A8%EB%8B%A4%EA%B3%B5%EC%A6%9D%EC%97%90%EC%A2%8B%EC%9D%80%EC%9D%8C%EC%8B%9D</t>
+  </si>
+  <si>
+    <t>골다공증에좋은음식 TOP7 골감소증 전후로 알아둘것</t>
+  </si>
+  <si>
+    <t>돌선물</t>
+  </si>
+  <si>
+    <t>돌선물추천</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/bongbong/contents/internal/909177147829824?areacode=itb_bas%2Af_challenge&amp;query=%EB%8F%8C%EC%84%A0%EB%AC%BC</t>
+  </si>
+  <si>
+    <t>돌선물 돌선물추천 두뇌발달 면역력 한번에 챙기는 올로메가베이비스마트</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/bongbong/contents/internal/909176406502432?areacode=itb_bas%2Af_challenge&amp;query=%EC%9C%A0%EC%95%84%EC%98%81%EC%96%91%EC%A0%9C</t>
+  </si>
+  <si>
+    <t>유아영양제 유아비타민 유아오메가3 성분 선택 기준</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/ryuae4/contents/internal/909175525411872?areacode=ink*a&amp;query=%EC%97%BC%EC%A6%9D%EC%88%98%EC%B9%98</t>
+  </si>
+  <si>
+    <t>염증수치 높을때 증상 및 관리방법 확인하세요</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/allcllrp/contents/internal/909511814557504?areacode=itb_bas%2Af_challenge&amp;query=%ED%98%88%EC%95%95%EB%82%AE%EC%B6%94%EB%8A%94%EB%B2%95</t>
+  </si>
+  <si>
+    <t>혈압낮추는음식 혈압낮추는법!</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/allcllrp/contents/internal/909931273572288?areacode=ink*a&amp;query=%ED%9D%91%EC%97%BC%EC%86%8C%EC%A7%84%EC%95%A1%ED%9A%A8%EB%8A%A5</t>
+  </si>
+  <si>
+    <t>염소즙 흑염소진액효능 팩트 체크</t>
+  </si>
+  <si>
+    <t>울금효능 강황 커큐민 '이렇게' 드셔야 해요 (시간낭비X)</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/binaida/contents/internal/907207386611104?areacode=itb_bas%2Af_challenge&amp;query=%ED%98%88%EB%8B%B9%EB%82%AE%EC%B6%94%EB%8A%94%EB%B2%95</t>
+  </si>
+  <si>
+    <t>혈당낮추는법 성공하는 영양제 선택 기준</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/eunchoda/contents/internal/910931746709248?areacode=ink*a&amp;query=%EA%B3%A0%ED%98%88%EC%95%95%EC%A6%9D%EC%83%81</t>
+  </si>
+  <si>
+    <t>고혈압증상, 그냥 피곤한 줄 알았는데 원인이 따로?</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/allcllrp/contents/internal/911456077590592?areacode=itb_bas%2Af_challenge&amp;query=%EC%95%84%EA%B8%B0%EC%84%B1%EC%9E%A5%EB%B0%9C%EB%8B%AC</t>
+  </si>
+  <si>
+    <t>아기성장발달 언제일까</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/binaida/contents/internal/911617314861280?areacode=ink*a&amp;query=%EB%AA%B8%EC%86%8D%EC%97%BC%EC%A6%9D%EC%A0%9C%EA%B1%B0</t>
+  </si>
+  <si>
+    <t>몸속염증제거 실패? 만성편도염 등 만성염증증상 관리하려면</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/drtella/contents/internal/911708321075424?areacode=itb_bas%2Af_challenge&amp;query=%EA%B0%84%EA%B8%B0%EB%8A%A5%EA%B0%9C%EC%84%A0%EC%A0%9C</t>
+  </si>
+  <si>
+    <t>간기능개선제 간기능저하 막는 간보호제 활용법</t>
+  </si>
+  <si>
+    <t>https://in.naver.com/eunchoda/contents/internal/910932723478848?areacode=ink*a&amp;query=%EB%B9%88%ED%98%88%EC%97%90%EC%A2%8B%EC%9D%80%EC%9D%8C%EC%8B%9D</t>
+  </si>
+  <si>
+    <t>빈혈에좋은음식 바꾸니 ?빈혈증상, 빈혈원인 !</t>
   </si>
 </sst>
 </file>
@@ -477,7 +816,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38551976-6904-4A88-95FF-2CB19913CAF8}">
-  <dimension ref="A1:C5"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.25" bestFit="1" customWidth="1"/>
@@ -486,57 +826,750 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>111</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>83</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>83</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>120</v>
+      </c>
+      <c r="C8" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" t="s">
+        <v>120</v>
+      </c>
+      <c r="C9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
+        <v>120</v>
+      </c>
+      <c r="C10" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" t="s">
+        <v>120</v>
+      </c>
+      <c r="C11" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" t="s">
+        <v>95</v>
+      </c>
+      <c r="C12" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" t="s">
+        <v>95</v>
+      </c>
+      <c r="C13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" t="s">
+        <v>92</v>
+      </c>
+      <c r="C14" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" t="s">
+        <v>92</v>
+      </c>
+      <c r="C15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" t="s">
+        <v>118</v>
+      </c>
+      <c r="C16" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" t="s">
+        <v>126</v>
+      </c>
+      <c r="C17" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" t="s">
+        <v>126</v>
+      </c>
+      <c r="C18" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" t="s">
+        <v>126</v>
+      </c>
+      <c r="C19" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>103</v>
+      </c>
+      <c r="B20" t="s">
+        <v>105</v>
+      </c>
+      <c r="C20" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>104</v>
+      </c>
+      <c r="B21" t="s">
+        <v>105</v>
+      </c>
+      <c r="C21" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" t="s">
+        <v>107</v>
+      </c>
+      <c r="C22" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" t="s">
+        <v>107</v>
+      </c>
+      <c r="C23" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24" t="s">
+        <v>107</v>
+      </c>
+      <c r="C24" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" t="s">
+        <v>91</v>
+      </c>
+      <c r="C25" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" t="s">
+        <v>91</v>
+      </c>
+      <c r="C26" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" t="s">
+        <v>122</v>
+      </c>
+      <c r="C27" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" t="s">
+        <v>122</v>
+      </c>
+      <c r="C28" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>36</v>
+      </c>
+      <c r="B29" t="s">
+        <v>122</v>
+      </c>
+      <c r="C29" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>37</v>
+      </c>
+      <c r="B30" t="s">
+        <v>93</v>
+      </c>
+      <c r="C30" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>2</v>
+      </c>
+      <c r="B31" t="s">
+        <v>93</v>
+      </c>
+      <c r="C31" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>38</v>
+      </c>
+      <c r="B32" t="s">
+        <v>8</v>
+      </c>
+      <c r="C32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>40</v>
+      </c>
+      <c r="B34" t="s">
+        <v>8</v>
+      </c>
+      <c r="C34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>41</v>
+      </c>
+      <c r="B35" t="s">
+        <v>116</v>
+      </c>
+      <c r="C35" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>42</v>
+      </c>
+      <c r="B36" t="s">
+        <v>116</v>
+      </c>
+      <c r="C36" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>43</v>
+      </c>
+      <c r="B37" t="s">
+        <v>84</v>
+      </c>
+      <c r="C37" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>44</v>
+      </c>
+      <c r="B38" t="s">
+        <v>84</v>
+      </c>
+      <c r="C38" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>45</v>
+      </c>
+      <c r="B39" t="s">
+        <v>84</v>
+      </c>
+      <c r="C39" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>46</v>
+      </c>
+      <c r="B40" t="s">
+        <v>73</v>
+      </c>
+      <c r="C40" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>47</v>
+      </c>
+      <c r="B41" t="s">
+        <v>73</v>
+      </c>
+      <c r="C41" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>48</v>
+      </c>
+      <c r="B42" t="s">
+        <v>75</v>
+      </c>
+      <c r="C42" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>49</v>
+      </c>
+      <c r="B43" t="s">
+        <v>75</v>
+      </c>
+      <c r="C43" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>50</v>
+      </c>
+      <c r="B44" t="s">
+        <v>75</v>
+      </c>
+      <c r="C44" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>69</v>
+      </c>
+      <c r="B45" t="s">
+        <v>77</v>
+      </c>
+      <c r="C45" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>70</v>
+      </c>
+      <c r="B46" t="s">
+        <v>77</v>
+      </c>
+      <c r="C46" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>71</v>
+      </c>
+      <c r="B47" t="s">
+        <v>77</v>
+      </c>
+      <c r="C47" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>72</v>
+      </c>
+      <c r="B48" t="s">
+        <v>77</v>
+      </c>
+      <c r="C48" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" t="s">
+        <v>97</v>
+      </c>
+      <c r="C49" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" t="s">
+        <v>97</v>
+      </c>
+      <c r="C50" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>53</v>
+      </c>
+      <c r="B51" t="s">
+        <v>79</v>
+      </c>
+      <c r="C51" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>81</v>
+      </c>
+      <c r="B52" t="s">
+        <v>79</v>
+      </c>
+      <c r="C52" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>54</v>
+      </c>
+      <c r="B53" t="s">
         <v>10</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C53" t="s">
         <v>11</v>
       </c>
-      <c r="C5" t="s">
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>55</v>
+      </c>
+      <c r="B54" t="s">
+        <v>10</v>
+      </c>
+      <c r="C54" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>56</v>
+      </c>
+      <c r="B55" t="s">
+        <v>99</v>
+      </c>
+      <c r="C55" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>57</v>
+      </c>
+      <c r="B56" t="s">
+        <v>99</v>
+      </c>
+      <c r="C56" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>58</v>
+      </c>
+      <c r="B57" t="s">
         <v>12</v>
+      </c>
+      <c r="C57" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>59</v>
+      </c>
+      <c r="B58" t="s">
+        <v>12</v>
+      </c>
+      <c r="C58" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>60</v>
+      </c>
+      <c r="B59" t="s">
+        <v>85</v>
+      </c>
+      <c r="C59" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>61</v>
+      </c>
+      <c r="B60" t="s">
+        <v>85</v>
+      </c>
+      <c r="C60" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>82</v>
+      </c>
+      <c r="B61" t="s">
+        <v>109</v>
+      </c>
+      <c r="C61" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>62</v>
+      </c>
+      <c r="B62" t="s">
+        <v>101</v>
+      </c>
+      <c r="C62" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>63</v>
+      </c>
+      <c r="B63" t="s">
+        <v>101</v>
+      </c>
+      <c r="C63" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>64</v>
+      </c>
+      <c r="B64" t="s">
+        <v>86</v>
+      </c>
+      <c r="C64" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>65</v>
+      </c>
+      <c r="B65" t="s">
+        <v>86</v>
+      </c>
+      <c r="C65" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>66</v>
+      </c>
+      <c r="B66" t="s">
+        <v>124</v>
+      </c>
+      <c r="C66" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>67</v>
+      </c>
+      <c r="B67" t="s">
+        <v>124</v>
+      </c>
+      <c r="C67" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>68</v>
+      </c>
+      <c r="B68" t="s">
+        <v>124</v>
+      </c>
+      <c r="C68" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>